<commit_message>
Add % of Total row to Sheet 7's Tier x Aging Schedule cross-tab
Each of the two tables (Units, Value) now gets a "% of Total" row
below the Total row, showing what share of the grand total each
exit-urgency column represents -- e.g. Long runway (FW28+) is 65.5%
of units but 74.1% of value, Not on FW27 Plan is 24.1% of units but
only 8.9% of value (its stock skews toward lower-value SKUs).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AbydMwYNKodhpRSt4oHY6f
</commit_message>
<xml_diff>
--- a/data/inventory_analysis/Project_Bob_Sell_Down_Priority_11092026.xlsx
+++ b/data/inventory_analysis/Project_Bob_Sell_Down_Priority_11092026.xlsx
@@ -22,8 +22,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="6">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0&quot;%&quot;"/>
+  </numFmts>
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -52,6 +54,11 @@
       <name val="Arial"/>
       <b val="1"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="FF555555"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -79,7 +86,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -99,6 +106,8 @@
     </xf>
     <xf numFmtId="3" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -24878,7 +24887,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -25206,98 +25215,98 @@
         <v>527963</v>
       </c>
     </row>
-    <row r="17" ht="60" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>% of Total</t>
+        </is>
+      </c>
+      <c r="B16" s="14" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="C16" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="14" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E16" s="14" t="n">
+        <v>65.5</v>
+      </c>
+      <c r="F16" s="14" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="G16" s="14" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="H16" s="14" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18" ht="60" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>Value below mixes bases (Target RRP for Sheets 2-3's columns, Historical ASP for "Not on FW27 Plan" per REG-INV-015) -- read each cell's own column for what it means, don't sum across the RRP and ASP columns as if they were the same currency of estimate. Cells with no price source (REG-INV-016) show as 0 here, not blank -- cross-reference the Units table above for what's actually being undercounted.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="1" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
         <is>
           <t>Value (mixed basis — see note above), SEK</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="10" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
         <is>
           <t>Portfolio Tier</t>
         </is>
       </c>
-      <c r="B20" s="10" t="inlineStr">
+      <c r="B21" s="10" t="inlineStr">
         <is>
           <t>Exiting FW27 (last season offered)</t>
         </is>
       </c>
-      <c r="C20" s="10" t="inlineStr">
+      <c r="C21" s="10" t="inlineStr">
         <is>
           <t>Exiting FW27 or SS28 (ambiguous — treat as near-term)</t>
         </is>
       </c>
-      <c r="D20" s="10" t="inlineStr">
+      <c r="D21" s="10" t="inlineStr">
         <is>
           <t>One season left (exits after SS28)</t>
         </is>
       </c>
-      <c r="E20" s="10" t="inlineStr">
+      <c r="E21" s="10" t="inlineStr">
         <is>
           <t>Long runway (continues through FW28+)</t>
         </is>
       </c>
-      <c r="F20" s="10" t="inlineStr">
+      <c r="F21" s="10" t="inlineStr">
         <is>
           <t>Pending Review (exit season = REVIEW)</t>
         </is>
       </c>
-      <c r="G20" s="10" t="inlineStr">
+      <c r="G21" s="10" t="inlineStr">
         <is>
           <t>Not on FW27 Plan</t>
         </is>
       </c>
-      <c r="H20" s="10" t="inlineStr">
+      <c r="H21" s="10" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>Hero + Near-Hero</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C21" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D21" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" s="6" t="n">
-        <v>117506600</v>
-      </c>
-      <c r="F21" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G21" s="6" t="n">
-        <v>1656580</v>
-      </c>
-      <c r="H21" s="11" t="n">
-        <v>119163180</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Workhorse + Harvest</t>
+          <t>Hero + Near-Hero</t>
         </is>
       </c>
       <c r="B22" s="6" t="n">
-        <v>4007300</v>
+        <v>0</v>
       </c>
       <c r="C22" s="6" t="n">
         <v>0</v>
@@ -25306,26 +25315,26 @@
         <v>0</v>
       </c>
       <c r="E22" s="6" t="n">
-        <v>227551200</v>
+        <v>117506600</v>
       </c>
       <c r="F22" s="6" t="n">
-        <v>937900</v>
+        <v>0</v>
       </c>
       <c r="G22" s="6" t="n">
-        <v>26393822</v>
+        <v>1656580</v>
       </c>
       <c r="H22" s="11" t="n">
-        <v>258890222</v>
+        <v>119163180</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Problem Child</t>
+          <t>Workhorse + Harvest</t>
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>4382300</v>
+        <v>4007300</v>
       </c>
       <c r="C23" s="6" t="n">
         <v>0</v>
@@ -25334,78 +25343,78 @@
         <v>0</v>
       </c>
       <c r="E23" s="6" t="n">
-        <v>22380900</v>
+        <v>227551200</v>
       </c>
       <c r="F23" s="6" t="n">
-        <v>0</v>
+        <v>937900</v>
       </c>
       <c r="G23" s="6" t="n">
-        <v>6630318</v>
+        <v>26393822</v>
       </c>
       <c r="H23" s="11" t="n">
-        <v>33393518</v>
+        <v>258890222</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>New / Test</t>
+          <t>Problem Child</t>
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>48077300</v>
+        <v>4382300</v>
       </c>
       <c r="C24" s="6" t="n">
-        <v>7147800</v>
+        <v>0</v>
       </c>
       <c r="D24" s="6" t="n">
-        <v>14497300</v>
+        <v>0</v>
       </c>
       <c r="E24" s="6" t="n">
-        <v>161517500</v>
+        <v>22380900</v>
       </c>
       <c r="F24" s="6" t="n">
-        <v>10367500</v>
+        <v>0</v>
       </c>
       <c r="G24" s="6" t="n">
-        <v>37889345</v>
+        <v>6630318</v>
       </c>
       <c r="H24" s="11" t="n">
-        <v>279496745</v>
+        <v>33393518</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Thin / Immaterial</t>
+          <t>New / Test</t>
         </is>
       </c>
       <c r="B25" s="6" t="n">
-        <v>0</v>
+        <v>48077300</v>
       </c>
       <c r="C25" s="6" t="n">
-        <v>0</v>
+        <v>7147800</v>
       </c>
       <c r="D25" s="6" t="n">
-        <v>11208400</v>
+        <v>14497300</v>
       </c>
       <c r="E25" s="6" t="n">
-        <v>86610350</v>
+        <v>161517500</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>33853750</v>
+        <v>10367500</v>
       </c>
       <c r="G25" s="6" t="n">
-        <v>1741634</v>
+        <v>37889345</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>133414134</v>
+        <v>279496745</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Exited</t>
+          <t>Thin / Immaterial</t>
         </is>
       </c>
       <c r="B26" s="6" t="n">
@@ -25415,25 +25424,25 @@
         <v>0</v>
       </c>
       <c r="D26" s="6" t="n">
-        <v>0</v>
+        <v>11208400</v>
       </c>
       <c r="E26" s="6" t="n">
-        <v>1457100</v>
+        <v>86610350</v>
       </c>
       <c r="F26" s="6" t="n">
-        <v>1175700</v>
+        <v>33853750</v>
       </c>
       <c r="G26" s="6" t="n">
-        <v>561829</v>
+        <v>1741634</v>
       </c>
       <c r="H26" s="11" t="n">
-        <v>3194629</v>
+        <v>133414134</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Clearance — Ex China/Zalando</t>
+          <t>Exited</t>
         </is>
       </c>
       <c r="B27" s="6" t="n">
@@ -25446,81 +25455,137 @@
         <v>0</v>
       </c>
       <c r="E27" s="6" t="n">
-        <v>0</v>
+        <v>1457100</v>
       </c>
       <c r="F27" s="6" t="n">
-        <v>0</v>
+        <v>1175700</v>
       </c>
       <c r="G27" s="6" t="n">
-        <v>1023629</v>
+        <v>561829</v>
       </c>
       <c r="H27" s="11" t="n">
-        <v>1023629</v>
+        <v>3194629</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Not in tiering workbook</t>
+          <t>Clearance — Ex China/Zalando</t>
         </is>
       </c>
       <c r="B28" s="6" t="n">
         <v>0</v>
       </c>
       <c r="C28" s="6" t="n">
-        <v>904800</v>
+        <v>0</v>
       </c>
       <c r="D28" s="6" t="n">
         <v>0</v>
       </c>
       <c r="E28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="6" t="n">
+        <v>1023629</v>
+      </c>
+      <c r="H28" s="11" t="n">
+        <v>1023629</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Not in tiering workbook</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="6" t="n">
+        <v>904800</v>
+      </c>
+      <c r="D29" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="6" t="n">
         <v>13679000</v>
       </c>
-      <c r="F28" s="6" t="n">
+      <c r="F29" s="6" t="n">
         <v>7922500</v>
       </c>
-      <c r="G28" s="6" t="n">
+      <c r="G29" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="H28" s="11" t="n">
+      <c r="H29" s="11" t="n">
         <v>22506300</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="12" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="12" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B29" s="11" t="n">
+      <c r="B30" s="11" t="n">
         <v>56466900</v>
       </c>
-      <c r="C29" s="11" t="n">
+      <c r="C30" s="11" t="n">
         <v>8052600</v>
       </c>
-      <c r="D29" s="11" t="n">
+      <c r="D30" s="11" t="n">
         <v>25705700</v>
       </c>
-      <c r="E29" s="11" t="n">
+      <c r="E30" s="11" t="n">
         <v>630702650</v>
       </c>
-      <c r="F29" s="11" t="n">
+      <c r="F30" s="11" t="n">
         <v>54257350</v>
       </c>
-      <c r="G29" s="11" t="n">
+      <c r="G30" s="11" t="n">
         <v>75897156</v>
       </c>
-      <c r="H29" s="11" t="n">
+      <c r="H30" s="11" t="n">
         <v>851082356</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="13" t="inlineStr">
+        <is>
+          <t>% of Total</t>
+        </is>
+      </c>
+      <c r="B31" s="14" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="C31" s="14" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D31" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="E31" s="14" t="n">
+        <v>74.09999999999999</v>
+      </c>
+      <c r="F31" s="14" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="G31" s="14" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="H31" s="14" t="n">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
+    <mergeCell ref="A18:H18"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A19:H19"/>
+    <mergeCell ref="A20:H20"/>
     <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A17:H17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>